<commit_message>
DC Jack Cable link update in Client BOM @basit-eSpark FYI
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
+++ b/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20408"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.2\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83995EF0-721A-46C9-88BE-7247FFE2CE1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -481,20 +480,32 @@
     <t>Peripheral</t>
   </si>
   <si>
-    <t>USB DC 2.0*0.5mm Charging Cable for Mini S530 Smallest Invisible Wireless Bluetooth Earbuds Earphones Headphones Headset</t>
-  </si>
-  <si>
     <t>TC2030-CTX-NL 6-Pin “No Legs” Cable with 10-pin micro-connector for Cortex processors</t>
   </si>
   <si>
     <t>Tag Connect</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2M 1M 0.5M USB Port to 2.0*0.6mm 2.5*0.7mm 3.5*1.35mm 4.0*1.7mm 5.5*2.1mm 2.5mm x 0.7mm 5V DC Barrel Jack Power Cable Connector </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Color: 2.0 X 0.6mm)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,19 +521,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -581,8 +579,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -597,18 +602,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF03A4CB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -623,15 +622,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -656,52 +646,10 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -750,117 +698,65 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1148,13 +1044,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
@@ -1169,1101 +1065,1073 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="5" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="23">
+      <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="7">
         <v>6</v>
       </c>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="23">
+      <c r="B4" s="11">
         <f t="shared" ref="B4:B30" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="I4" s="18" t="s">
+      <c r="I4" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="J4" s="17">
-        <v>1</v>
-      </c>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
+      <c r="J4" s="9">
+        <v>1</v>
+      </c>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="23">
+      <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="J5" s="15">
-        <v>1</v>
-      </c>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
+      <c r="J5" s="7">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
     </row>
     <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="23">
+      <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I6" s="18" t="s">
+      <c r="I6" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J6" s="17">
-        <v>1</v>
-      </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
+      <c r="J6" s="9">
+        <v>1</v>
+      </c>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="23">
+      <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="7">
         <v>2</v>
       </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="23">
+      <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="I8" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="J8" s="17">
-        <v>1</v>
-      </c>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
+      <c r="J8" s="9">
+        <v>1</v>
+      </c>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="23">
+      <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="7">
         <v>2</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="23">
+      <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28" t="s">
+      <c r="H10" s="14"/>
+      <c r="I10" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="14">
         <v>4</v>
       </c>
-      <c r="K10" s="27"/>
-      <c r="L10" s="29" t="s">
+      <c r="K10" s="14"/>
+      <c r="L10" s="16" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="23">
+      <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="J11" s="15">
-        <v>1</v>
-      </c>
-      <c r="K11" s="30" t="s">
+      <c r="J11" s="7">
+        <v>1</v>
+      </c>
+      <c r="K11" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="L11" s="15"/>
+      <c r="L11" s="7"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="23">
+      <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="G12" s="28" t="s">
+      <c r="G12" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="H12" s="27"/>
-      <c r="I12" s="28" t="s">
+      <c r="H12" s="14"/>
+      <c r="I12" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="J12" s="27">
-        <v>1</v>
-      </c>
-      <c r="K12" s="27"/>
-      <c r="L12" s="29" t="s">
+      <c r="J12" s="14">
+        <v>1</v>
+      </c>
+      <c r="K12" s="14"/>
+      <c r="L12" s="16" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="23">
+      <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="27" t="s">
+      <c r="C13" s="12"/>
+      <c r="D13" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="28"/>
-      <c r="F13" s="27" t="s">
+      <c r="E13" s="15"/>
+      <c r="F13" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="27">
-        <v>1</v>
-      </c>
-      <c r="K13" s="27"/>
-      <c r="L13" s="29" t="s">
+      <c r="G13" s="15"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="14">
+        <v>1</v>
+      </c>
+      <c r="K13" s="14"/>
+      <c r="L13" s="16" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="23">
+      <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="I14" s="18" t="s">
+      <c r="I14" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="J14" s="17">
-        <v>1</v>
-      </c>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
+      <c r="J14" s="9">
+        <v>1</v>
+      </c>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
     </row>
     <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="23">
+      <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="I15" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="J15" s="15">
-        <v>1</v>
-      </c>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
+      <c r="J15" s="7">
+        <v>1</v>
+      </c>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="23">
+      <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="H16" s="17" t="s">
+      <c r="H16" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I16" s="18" t="s">
+      <c r="I16" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="J16" s="17">
+      <c r="J16" s="9">
         <v>6</v>
       </c>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
     </row>
     <row r="17" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="23">
+      <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="I17" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="J17" s="15">
-        <v>1</v>
-      </c>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
+      <c r="J17" s="7">
+        <v>1</v>
+      </c>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
     </row>
     <row r="18" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="23">
+      <c r="B18" s="11">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H18" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I18" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J18" s="17">
-        <v>1</v>
-      </c>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
+      <c r="J18" s="9">
+        <v>1</v>
+      </c>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="23">
+      <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="16" t="s">
+      <c r="G19" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="H19" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="I19" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="J19" s="15">
-        <v>1</v>
-      </c>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
+      <c r="J19" s="7">
+        <v>1</v>
+      </c>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="23">
+      <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="G20" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I20" s="18" t="s">
+      <c r="I20" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="J20" s="17">
-        <v>1</v>
-      </c>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
+      <c r="J20" s="9">
+        <v>1</v>
+      </c>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="23">
+      <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="E21" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="F21" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="H21" s="15" t="s">
+      <c r="H21" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="I21" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="J21" s="15">
+      <c r="J21" s="7">
         <v>2</v>
       </c>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="23">
+      <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H22" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="I22" s="18" t="s">
+      <c r="I22" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J22" s="17">
-        <v>1</v>
-      </c>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
+      <c r="J22" s="9">
+        <v>1</v>
+      </c>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
     </row>
     <row r="23" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="23">
+      <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="16" t="s">
+      <c r="E23" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="G23" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="H23" s="15" t="s">
+      <c r="H23" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="I23" s="18" t="s">
+      <c r="I23" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J23" s="15">
-        <v>1</v>
-      </c>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
+      <c r="J23" s="7">
+        <v>1</v>
+      </c>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="23">
+      <c r="B24" s="11">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="H24" s="17" t="s">
+      <c r="H24" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="I24" s="18" t="s">
+      <c r="I24" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J24" s="17">
-        <v>1</v>
-      </c>
-      <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
+      <c r="J24" s="9">
+        <v>1</v>
+      </c>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
     </row>
     <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="23">
+      <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="H25" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="I25" s="18" t="s">
+      <c r="I25" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J25" s="15">
-        <v>1</v>
-      </c>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
+      <c r="J25" s="7">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
     </row>
     <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="23">
+      <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C26" s="25" t="s">
+      <c r="C26" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G26" s="18" t="s">
+      <c r="G26" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="I26" s="18" t="s">
+      <c r="I26" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J26" s="17">
-        <v>1</v>
-      </c>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
+      <c r="J26" s="9">
+        <v>1</v>
+      </c>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="23">
+      <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="E27" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="F27" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="H27" s="15" t="s">
+      <c r="H27" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="I27" s="18" t="s">
+      <c r="I27" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J27" s="15">
-        <v>1</v>
-      </c>
-      <c r="K27" s="15"/>
-      <c r="L27" s="15"/>
+      <c r="J27" s="7">
+        <v>1</v>
+      </c>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
     </row>
     <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="23">
+      <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="17" t="s">
+      <c r="C28" s="13"/>
+      <c r="D28" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G28" s="18" t="s">
+      <c r="G28" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="I28" s="18" t="s">
+      <c r="I28" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J28" s="17">
-        <v>1</v>
-      </c>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
+      <c r="J28" s="9">
+        <v>1</v>
+      </c>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
     </row>
     <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="23">
+      <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="F29" s="15" t="s">
+      <c r="F29" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="H29" s="15" t="s">
+      <c r="H29" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="I29" s="18" t="s">
+      <c r="I29" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J29" s="15">
-        <v>1</v>
-      </c>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
+      <c r="J29" s="7">
+        <v>1</v>
+      </c>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="23">
+      <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="25" t="s">
+      <c r="C30" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="H30" s="17" t="s">
+      <c r="H30" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="I30" s="18" t="s">
+      <c r="I30" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J30" s="17">
-        <v>1</v>
-      </c>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
+      <c r="J30" s="9">
+        <v>1</v>
+      </c>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
     </row>
     <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="23">
+      <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="24" t="s">
+      <c r="C31" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F31" s="15" t="s">
+      <c r="F31" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G31" s="16" t="s">
+      <c r="G31" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="H31" s="15" t="s">
+      <c r="H31" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="I31" s="18" t="s">
+      <c r="I31" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="J31" s="15">
-        <v>1</v>
-      </c>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-    </row>
-    <row r="32" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J31" s="7">
+        <v>1</v>
+      </c>
+      <c r="K31" s="7"/>
+      <c r="L31" s="7"/>
+    </row>
+    <row r="32" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="23">
+      <c r="B32" s="11">
         <f t="shared" ref="B32:B33" si="1">ROW(B32) - ROW($B$2)</f>
         <v>30</v>
       </c>
-      <c r="C32" s="31" t="s">
+      <c r="C32" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="F32" s="15" t="s">
+      <c r="D32" s="7"/>
+      <c r="E32" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H32" s="15" t="s">
+      <c r="H32" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="I32" s="16" t="s">
+      <c r="I32" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="J32" s="15"/>
-      <c r="K32" s="30" t="s">
+      <c r="J32" s="7"/>
+      <c r="K32" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="L32" s="15"/>
+      <c r="L32" s="7"/>
     </row>
     <row r="33" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="23">
+      <c r="B33" s="11">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="C33" s="31" t="s">
+      <c r="C33" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="D33" s="15"/>
-      <c r="E33" s="16" t="s">
+      <c r="D33" s="7"/>
+      <c r="E33" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="J33" s="7"/>
+      <c r="K33" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="F33" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="I33" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="J33" s="15"/>
-      <c r="K33" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="L33" s="15"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="19"/>
-    </row>
-    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="1"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="20"/>
+      <c r="L33" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K11" r:id="rId1" xr:uid="{EB16CAE9-A630-49E2-B4EB-9E498E44D463}"/>
-    <hyperlink ref="K32" r:id="rId2" xr:uid="{81BDAFE3-2DB7-457C-95AE-A927BB5269FC}"/>
-    <hyperlink ref="K33" r:id="rId3" xr:uid="{64931943-BE44-4525-BA6B-29B5755EA863}"/>
+    <hyperlink ref="K11" r:id="rId1"/>
+    <hyperlink ref="K33" r:id="rId2"/>
+    <hyperlink ref="K32" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>

</xml_diff>

<commit_message>
#11 Completed and Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
+++ b/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20412"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.2\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.2\Project Outputs for BLE_product-v1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D295DD4D-8508-41DD-A02D-3B79D555000E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="153">
   <si>
     <t>#</t>
   </si>
@@ -201,7 +202,7 @@
     <t>RES 4.7K OHM 1% 1/20W 0201</t>
   </si>
   <si>
-    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+    <t>3.35mm 2.5mm Oval button 50mA Brick nogging 4.2mm 180gf 12V SMD Tactile Switches ROHS</t>
   </si>
   <si>
     <t>IC REG BOOST 5V 1A 9WLCSP</t>
@@ -255,256 +256,235 @@
     <t>Sensor-Pads 0.5mm Dia</t>
   </si>
   <si>
+    <t>IND-0806</t>
+  </si>
+  <si>
+    <t>XL-1010RGBC-WS2812B</t>
+  </si>
+  <si>
+    <t>Res-0201</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>TSA016A2518A</t>
+  </si>
+  <si>
+    <t>WLCSP-9 (1.22x1.22)</t>
+  </si>
+  <si>
+    <t>WLP-6(0.83x1.24)</t>
+  </si>
+  <si>
+    <t>X2-SON-4(1x1)</t>
+  </si>
+  <si>
+    <t>DFN-6-EP(2x2)</t>
+  </si>
+  <si>
+    <t>DSBGA-9 (1.651x1.61)</t>
+  </si>
+  <si>
+    <t>EYSHSNZWZ</t>
+  </si>
+  <si>
+    <t>X-LLGA-3</t>
+  </si>
+  <si>
+    <t>14-LGA (2.5x3)</t>
+  </si>
+  <si>
+    <t>12-WLCSP (1.56x1.56)</t>
+  </si>
+  <si>
+    <t>Manufacturer Part Number</t>
+  </si>
+  <si>
+    <t>CC0201KRX5R6BB104</t>
+  </si>
+  <si>
+    <t>CL05A106MP5NUNC</t>
+  </si>
+  <si>
+    <t>CC0603MRX5R6BB226</t>
+  </si>
+  <si>
+    <t>CC0201MRX5R6BB105</t>
+  </si>
+  <si>
+    <t>CC0201MRX5R6BB225</t>
+  </si>
+  <si>
+    <t>CC0201MRX5R7BB105</t>
+  </si>
+  <si>
+    <t>Sensor Pads</t>
+  </si>
+  <si>
+    <t>1286AS-H-R47M=P2</t>
+  </si>
+  <si>
+    <t>RC0201JR-0710KL</t>
+  </si>
+  <si>
+    <t>0201WMF2202TEE</t>
+  </si>
+  <si>
+    <t>0201WMF3302TEE</t>
+  </si>
+  <si>
+    <t>PE0402FRF470R01L</t>
+  </si>
+  <si>
+    <t>RC0201FR-075K1L</t>
+  </si>
+  <si>
+    <t>RC0201FR-074K7L</t>
+  </si>
+  <si>
+    <t>FAN48610UC50X</t>
+  </si>
+  <si>
+    <t>MAX16150AWT+</t>
+  </si>
+  <si>
+    <t>TLV73330PDQNR</t>
+  </si>
+  <si>
+    <t>FAN54120MP420X</t>
+  </si>
+  <si>
+    <t>BQ27426YZFR</t>
+  </si>
+  <si>
+    <t>NTNS3193NZT5G</t>
+  </si>
+  <si>
+    <t>BMI323</t>
+  </si>
+  <si>
+    <t>BMM150</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Yageo</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>Kyocera AVX</t>
+  </si>
+  <si>
+    <t>CW Switch Elec. Store</t>
+  </si>
+  <si>
+    <t>Murata</t>
+  </si>
+  <si>
+    <t>XINGLIGHT</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL</t>
+  </si>
+  <si>
+    <t>BZCN</t>
+  </si>
+  <si>
+    <t>ON Semiconductor / Fairchild</t>
+  </si>
+  <si>
+    <t>Analog Devices</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>ON Semiconductor</t>
+  </si>
+  <si>
+    <t>Taiyo Yuden</t>
+  </si>
+  <si>
+    <t>Bosch Sensortec</t>
+  </si>
+  <si>
+    <t>0.1uF</t>
+  </si>
+  <si>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>2.2uf</t>
+  </si>
+  <si>
+    <t>100uF</t>
+  </si>
+  <si>
+    <t>470nH</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>22K</t>
+  </si>
+  <si>
+    <t>33k</t>
+  </si>
+  <si>
+    <t>10mR</t>
+  </si>
+  <si>
+    <t>5.1K</t>
+  </si>
+  <si>
+    <t>4.7K</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>DNP</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>TC2030-IDC-NL_</t>
   </si>
   <si>
-    <t>IND-0806</t>
-  </si>
-  <si>
-    <t>XL-1010RGBC-WS2812B</t>
-  </si>
-  <si>
-    <t>Res-0201</t>
-  </si>
-  <si>
-    <t>Res-0402</t>
-  </si>
-  <si>
-    <t>EVQP7A01P</t>
-  </si>
-  <si>
-    <t>WLCSP-9 (1.22x1.22)</t>
-  </si>
-  <si>
-    <t>WLP-6(0.83x1.24)</t>
-  </si>
-  <si>
-    <t>X2-SON-4(1x1)</t>
-  </si>
-  <si>
-    <t>DFN-6-EP(2x2)</t>
-  </si>
-  <si>
-    <t>DSBGA-9 (1.651x1.61)</t>
-  </si>
-  <si>
-    <t>EYSHSNZWZ</t>
-  </si>
-  <si>
-    <t>X-LLGA-3</t>
-  </si>
-  <si>
-    <t>14-LGA (2.5x3)</t>
-  </si>
-  <si>
-    <t>12-WLCSP (1.56x1.56)</t>
-  </si>
-  <si>
-    <t>Manufacturer Part Number</t>
-  </si>
-  <si>
-    <t>CC0201KRX5R6BB104</t>
-  </si>
-  <si>
-    <t>CL05A106MP5NUNC</t>
-  </si>
-  <si>
-    <t>CC0603MRX5R6BB226</t>
-  </si>
-  <si>
-    <t>CC0201MRX5R6BB105</t>
-  </si>
-  <si>
-    <t>CC0201MRX5R6BB225</t>
-  </si>
-  <si>
-    <t>CC0201MRX5R7BB105</t>
-  </si>
-  <si>
-    <t>Sensor Pads</t>
-  </si>
-  <si>
-    <t>1286AS-H-R47M=P2</t>
-  </si>
-  <si>
-    <t>RC0201JR-0710KL</t>
-  </si>
-  <si>
-    <t>0201WMF2202TEE</t>
-  </si>
-  <si>
-    <t>0201WMF3302TEE</t>
-  </si>
-  <si>
-    <t>PE0402FRF470R01L</t>
-  </si>
-  <si>
-    <t>RC0201FR-075K1L</t>
-  </si>
-  <si>
-    <t>RC0201FR-074K7L</t>
-  </si>
-  <si>
-    <t>EVQ-P7A01P</t>
-  </si>
-  <si>
-    <t>FAN48610UC50X</t>
-  </si>
-  <si>
-    <t>MAX16150AWT+</t>
-  </si>
-  <si>
-    <t>TLV73330PDQNR</t>
-  </si>
-  <si>
-    <t>FAN54120MP420X</t>
-  </si>
-  <si>
-    <t>BQ27426YZFR</t>
-  </si>
-  <si>
-    <t>NTNS3193NZT5G</t>
-  </si>
-  <si>
-    <t>BMI323</t>
-  </si>
-  <si>
-    <t>BMM150</t>
-  </si>
-  <si>
-    <t>Manufacturer</t>
-  </si>
-  <si>
-    <t>Yageo</t>
-  </si>
-  <si>
-    <t>Samsung</t>
-  </si>
-  <si>
-    <t>Kyocera AVX</t>
-  </si>
-  <si>
-    <t>CW Switch Elec. Store</t>
-  </si>
-  <si>
-    <t>Murata</t>
-  </si>
-  <si>
-    <t>XINGLIGHT</t>
-  </si>
-  <si>
-    <t>UNI-ROYAL</t>
-  </si>
-  <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>ON Semiconductor / Fairchild</t>
-  </si>
-  <si>
-    <t>Analog Devices</t>
-  </si>
-  <si>
-    <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
-    <t>Taiyo Yuden</t>
-  </si>
-  <si>
-    <t>Bosch Sensortec</t>
-  </si>
-  <si>
-    <t>0.1uF</t>
-  </si>
-  <si>
-    <t>10uF</t>
-  </si>
-  <si>
-    <t>22uF</t>
-  </si>
-  <si>
-    <t>1uF</t>
-  </si>
-  <si>
-    <t>2.2uF</t>
-  </si>
-  <si>
-    <t>100uF</t>
-  </si>
-  <si>
-    <t>470nH</t>
-  </si>
-  <si>
-    <t>10K</t>
-  </si>
-  <si>
-    <t>22K</t>
-  </si>
-  <si>
-    <t>33k</t>
-  </si>
-  <si>
-    <t>10mR</t>
-  </si>
-  <si>
-    <t>5.1K</t>
-  </si>
-  <si>
-    <t>4.7K</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>DNP</t>
-  </si>
-  <si>
-    <t>Link</t>
-  </si>
-  <si>
     <t>Aliexpress</t>
   </si>
   <si>
     <t>Peripheral</t>
   </si>
   <si>
-    <t>TC2030-CTX-NL 6-Pin “No Legs” Cable with 10-pin micro-connector for Cortex processors</t>
-  </si>
-  <si>
-    <t>Tag Connect</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">2M 1M 0.5M USB Port to 2.0*0.6mm 2.5*0.7mm 3.5*1.35mm 4.0*1.7mm 5.5*2.1mm 2.5mm x 0.7mm 5V DC Barrel Jack Power Cable Connector </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(Color: 2.0 X 0.6mm)</t>
-    </r>
+    <t>2M 1M 0.5M USB Port to 2.0*0.6mm 2.5*0.7mm 3.5*1.35mm 4.0*1.7mm 5.5*2.1mm 2.5mm x 0.7mm 5V DC Barrel Jack Power Cable Connector (Color: 2.0 X 0.6mm)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -549,7 +529,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -557,7 +543,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -575,13 +561,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -607,7 +586,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -698,12 +677,64 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -740,23 +771,51 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1044,9 +1103,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1056,11 +1115,10 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1072,10 +1130,8 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1095,21 +1151,21 @@
         <v>70</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="15" t="s">
         <v>146</v>
       </c>
     </row>
@@ -1132,19 +1188,19 @@
         <v>71</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="J3" s="7">
+        <v>130</v>
+      </c>
+      <c r="J3" s="16">
         <v>6</v>
       </c>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1165,19 +1221,19 @@
         <v>72</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="J4" s="9">
-        <v>1</v>
-      </c>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
+        <v>131</v>
+      </c>
+      <c r="J4" s="17">
+        <v>1</v>
+      </c>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
     </row>
     <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -1198,19 +1254,19 @@
         <v>73</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="J5" s="7">
-        <v>1</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
+        <v>132</v>
+      </c>
+      <c r="J5" s="16">
+        <v>1</v>
+      </c>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
     </row>
     <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -1231,19 +1287,19 @@
         <v>71</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="J6" s="9">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
+        <v>133</v>
+      </c>
+      <c r="J6" s="17">
+        <v>1</v>
+      </c>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1264,19 +1320,19 @@
         <v>71</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="J7" s="7">
+        <v>134</v>
+      </c>
+      <c r="J7" s="16">
         <v>2</v>
       </c>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1300,16 +1356,16 @@
         <v>74</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="J8" s="9">
-        <v>1</v>
-      </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
+        <v>135</v>
+      </c>
+      <c r="J8" s="17">
+        <v>1</v>
+      </c>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1330,19 +1386,19 @@
         <v>71</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="J9" s="7">
+        <v>133</v>
+      </c>
+      <c r="J9" s="16">
         <v>2</v>
       </c>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -1353,28 +1409,28 @@
       <c r="C10" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="G10" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="s">
+      <c r="G10" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" s="19"/>
+      <c r="I10" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="21">
         <v>4</v>
       </c>
-      <c r="K10" s="14"/>
-      <c r="L10" s="16" t="s">
-        <v>149</v>
+      <c r="K10" s="18"/>
+      <c r="L10" s="24" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1399,18 +1455,18 @@
         <v>76</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="J11" s="7">
-        <v>1</v>
-      </c>
-      <c r="K11" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="L11" s="7"/>
+        <v>76</v>
+      </c>
+      <c r="J11" s="16">
+        <v>1</v>
+      </c>
+      <c r="K11" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="L11" s="18"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -1421,28 +1477,28 @@
       <c r="C12" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="G12" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="s">
+      <c r="G12" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="9"/>
+      <c r="I12" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="J12" s="14">
-        <v>1</v>
-      </c>
-      <c r="K12" s="14"/>
-      <c r="L12" s="16" t="s">
-        <v>149</v>
+      <c r="J12" s="21">
+        <v>1</v>
+      </c>
+      <c r="K12" s="18"/>
+      <c r="L12" s="24" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1452,22 +1508,22 @@
         <v>11</v>
       </c>
       <c r="C13" s="12"/>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="14">
-        <v>1</v>
-      </c>
-      <c r="K13" s="14"/>
-      <c r="L13" s="16" t="s">
+      <c r="E13" s="26"/>
+      <c r="F13" s="22" t="s">
         <v>149</v>
+      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="25">
+        <v>1</v>
+      </c>
+      <c r="K13" s="18"/>
+      <c r="L13" s="24" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1486,22 +1542,22 @@
         <v>52</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="J14" s="9">
-        <v>1</v>
-      </c>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
+        <v>136</v>
+      </c>
+      <c r="J14" s="17">
+        <v>1</v>
+      </c>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
@@ -1519,22 +1575,22 @@
         <v>53</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="J15" s="7">
-        <v>1</v>
-      </c>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
+        <v>79</v>
+      </c>
+      <c r="J15" s="16">
+        <v>1</v>
+      </c>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
@@ -1552,22 +1608,22 @@
         <v>54</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="J16" s="9">
+        <v>137</v>
+      </c>
+      <c r="J16" s="17">
         <v>6</v>
       </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -1585,22 +1641,22 @@
         <v>55</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="J17" s="7">
-        <v>1</v>
-      </c>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
+        <v>138</v>
+      </c>
+      <c r="J17" s="16">
+        <v>1</v>
+      </c>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
     </row>
     <row r="18" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -1618,22 +1674,22 @@
         <v>56</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="J18" s="9">
-        <v>1</v>
-      </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
+        <v>139</v>
+      </c>
+      <c r="J18" s="17">
+        <v>1</v>
+      </c>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
@@ -1651,22 +1707,22 @@
         <v>57</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="J19" s="7">
-        <v>1</v>
-      </c>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7"/>
+        <v>140</v>
+      </c>
+      <c r="J19" s="16">
+        <v>1</v>
+      </c>
+      <c r="K19" s="18"/>
+      <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -1684,22 +1740,22 @@
         <v>58</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="J20" s="9">
-        <v>1</v>
-      </c>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
+        <v>141</v>
+      </c>
+      <c r="J20" s="17">
+        <v>1</v>
+      </c>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
@@ -1717,24 +1773,24 @@
         <v>59</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="J21" s="7">
+        <v>142</v>
+      </c>
+      <c r="J21" s="16">
         <v>2</v>
       </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-    </row>
-    <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K21" s="18"/>
+      <c r="L21" s="18"/>
+    </row>
+    <row r="22" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1750,22 +1806,22 @@
         <v>60</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J22" s="9">
-        <v>1</v>
-      </c>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
+        <v>82</v>
+      </c>
+      <c r="J22" s="17">
+        <v>1</v>
+      </c>
+      <c r="K22" s="18"/>
+      <c r="L22" s="18"/>
     </row>
     <row r="23" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -1783,22 +1839,22 @@
         <v>61</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J23" s="7">
-        <v>1</v>
-      </c>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
+        <v>124</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="16">
+        <v>1</v>
+      </c>
+      <c r="K23" s="18"/>
+      <c r="L23" s="18"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -1816,22 +1872,22 @@
         <v>62</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J24" s="9">
-        <v>1</v>
-      </c>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
+        <v>108</v>
+      </c>
+      <c r="J24" s="17">
+        <v>1</v>
+      </c>
+      <c r="K24" s="18"/>
+      <c r="L24" s="18"/>
     </row>
     <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -1849,22 +1905,22 @@
         <v>63</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J25" s="7">
-        <v>1</v>
-      </c>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
+        <v>126</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="J25" s="16">
+        <v>1</v>
+      </c>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
     </row>
     <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -1882,22 +1938,22 @@
         <v>64</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J26" s="9">
-        <v>1</v>
-      </c>
-      <c r="K26" s="9"/>
-      <c r="L26" s="9"/>
+        <v>110</v>
+      </c>
+      <c r="J26" s="17">
+        <v>1</v>
+      </c>
+      <c r="K26" s="18"/>
+      <c r="L26" s="18"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -1915,22 +1971,22 @@
         <v>65</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J27" s="7">
-        <v>1</v>
-      </c>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
+        <v>126</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="J27" s="16">
+        <v>1</v>
+      </c>
+      <c r="K27" s="18"/>
+      <c r="L27" s="18"/>
     </row>
     <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
@@ -1946,22 +2002,22 @@
         <v>66</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J28" s="9">
-        <v>1</v>
-      </c>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
+        <v>88</v>
+      </c>
+      <c r="J28" s="17">
+        <v>1</v>
+      </c>
+      <c r="K28" s="18"/>
+      <c r="L28" s="18"/>
     </row>
     <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -1979,22 +2035,22 @@
         <v>67</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="I29" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J29" s="7">
-        <v>1</v>
-      </c>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
+        <v>127</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J29" s="16">
+        <v>1</v>
+      </c>
+      <c r="K29" s="18"/>
+      <c r="L29" s="18"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -2012,22 +2068,22 @@
         <v>68</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J30" s="9">
-        <v>1</v>
-      </c>
-      <c r="K30" s="9"/>
-      <c r="L30" s="9"/>
+        <v>113</v>
+      </c>
+      <c r="J30" s="17">
+        <v>1</v>
+      </c>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
     </row>
     <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -2045,95 +2101,95 @@
         <v>69</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J31" s="7">
-        <v>1</v>
-      </c>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
+        <v>129</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="J31" s="16">
+        <v>1</v>
+      </c>
+      <c r="K31" s="18"/>
+      <c r="L31" s="18"/>
     </row>
     <row r="32" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" ref="B32:B33" si="1">ROW(B32) - ROW($B$2)</f>
         <v>30</v>
       </c>
-      <c r="C32" s="18" t="s">
-        <v>152</v>
+      <c r="C32" s="28" t="s">
+        <v>151</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F32" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F32" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H32" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="I32" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="J32" s="7"/>
-      <c r="K32" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="L32" s="7"/>
-    </row>
-    <row r="33" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
+      <c r="J32" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+    </row>
+    <row r="33" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="C33" s="18" t="s">
-        <v>152</v>
+      <c r="C33" s="28" t="s">
+        <v>151</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="F33" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="H33" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="I33" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="J33" s="7"/>
-      <c r="K33" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="L33" s="7"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+    </row>
+    <row r="37" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="M37" s="28" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K11" r:id="rId1"/>
-    <hyperlink ref="K33" r:id="rId2"/>
-    <hyperlink ref="K32" r:id="rId3"/>
+    <hyperlink ref="K11" r:id="rId1" xr:uid="{03266B9D-911B-4550-9416-FC47FB8879C8}"/>
+    <hyperlink ref="J32" r:id="rId2" xr:uid="{D1E8C578-5D82-4E69-90F3-A5AB52CCB2B0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Tag Connect description fix in BOM #11
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
+++ b/Design Files/BLE_product-v1.2/Deliverables/BOM/BLE_product-v1.2.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20412"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.2\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\raafat-BLEproduct\Design Files\BLE_product-v1.2\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C6CB7E-951B-408A-9856-6FD350B6FBC5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,12 +18,12 @@
     <definedName name="LINK">Sheet1!$K$33</definedName>
     <definedName name="LinnKs">Sheet1!$K$33</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="155">
   <si>
     <t>#</t>
   </si>
@@ -485,13 +484,16 @@
     <t>2M 1M 0.5M USB Port to 2.0*0.6mm 2.5*0.7mm 3.5*1.35mm 4.0*1.7mm 5.5*2.1mm 2.5mm x 0.7mm 5V DC Barrel Jack Power Cable Connector (Color: 2.0 X 0.6mm)</t>
   </si>
   <si>
-    <t>link</t>
+    <t>TC2030-CTX 6-Pin Cable for ARM Cortex</t>
+  </si>
+  <si>
+    <t>Tag-Connect</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -870,9 +872,6 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -917,6 +916,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1204,7 +1206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1231,8 +1233,8 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1297,11 +1299,11 @@
       <c r="I3" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="J3" s="31">
+      <c r="J3" s="30">
         <v>6</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1333,8 +1335,8 @@
       <c r="J4" s="9">
         <v>1</v>
       </c>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
     </row>
     <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -1366,8 +1368,8 @@
       <c r="J5" s="7">
         <v>1</v>
       </c>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
     </row>
     <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -1399,8 +1401,8 @@
       <c r="J6" s="9">
         <v>1</v>
       </c>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1432,8 +1434,8 @@
       <c r="J7" s="7">
         <v>2</v>
       </c>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1465,8 +1467,8 @@
       <c r="J8" s="9">
         <v>1</v>
       </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1498,8 +1500,8 @@
       <c r="J9" s="7">
         <v>2</v>
       </c>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -1529,8 +1531,8 @@
       <c r="J10" s="15">
         <v>4</v>
       </c>
-      <c r="K10" s="26"/>
-      <c r="L10" s="27" t="s">
+      <c r="K10" s="25"/>
+      <c r="L10" s="26" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1564,10 +1566,10 @@
       <c r="J11" s="9">
         <v>1</v>
       </c>
-      <c r="K11" s="30" t="s">
+      <c r="K11" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="L11" s="26"/>
+      <c r="L11" s="25"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -1597,8 +1599,8 @@
       <c r="J12" s="15">
         <v>1</v>
       </c>
-      <c r="K12" s="26"/>
-      <c r="L12" s="27" t="s">
+      <c r="K12" s="25"/>
+      <c r="L12" s="26" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1619,11 +1621,11 @@
       <c r="G13" s="8"/>
       <c r="H13" s="7"/>
       <c r="I13" s="8"/>
-      <c r="J13" s="32">
-        <v>1</v>
-      </c>
-      <c r="K13" s="26"/>
-      <c r="L13" s="27" t="s">
+      <c r="J13" s="31">
+        <v>1</v>
+      </c>
+      <c r="K13" s="25"/>
+      <c r="L13" s="26" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1657,8 +1659,8 @@
       <c r="J14" s="9">
         <v>1</v>
       </c>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
     </row>
     <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
@@ -1690,8 +1692,8 @@
       <c r="J15" s="7">
         <v>1</v>
       </c>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
@@ -1723,8 +1725,8 @@
       <c r="J16" s="9">
         <v>6</v>
       </c>
-      <c r="K16" s="26"/>
-      <c r="L16" s="26"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
     </row>
     <row r="17" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -1756,8 +1758,8 @@
       <c r="J17" s="7">
         <v>1</v>
       </c>
-      <c r="K17" s="26"/>
-      <c r="L17" s="26"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
     </row>
     <row r="18" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -1789,8 +1791,8 @@
       <c r="J18" s="9">
         <v>1</v>
       </c>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
@@ -1822,8 +1824,8 @@
       <c r="J19" s="7">
         <v>1</v>
       </c>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -1855,8 +1857,8 @@
       <c r="J20" s="9">
         <v>1</v>
       </c>
-      <c r="K20" s="26"/>
-      <c r="L20" s="26"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
@@ -1888,8 +1890,8 @@
       <c r="J21" s="7">
         <v>2</v>
       </c>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="25"/>
     </row>
     <row r="22" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -1921,8 +1923,8 @@
       <c r="J22" s="9">
         <v>1</v>
       </c>
-      <c r="K22" s="26"/>
-      <c r="L22" s="26"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25"/>
     </row>
     <row r="23" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -1954,8 +1956,8 @@
       <c r="J23" s="7">
         <v>1</v>
       </c>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -1987,8 +1989,8 @@
       <c r="J24" s="9">
         <v>1</v>
       </c>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25"/>
     </row>
     <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -2020,8 +2022,8 @@
       <c r="J25" s="7">
         <v>1</v>
       </c>
-      <c r="K25" s="26"/>
-      <c r="L25" s="26"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
     </row>
     <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -2053,8 +2055,8 @@
       <c r="J26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -2086,8 +2088,8 @@
       <c r="J27" s="7">
         <v>1</v>
       </c>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
     </row>
     <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
@@ -2117,8 +2119,8 @@
       <c r="J28" s="9">
         <v>1</v>
       </c>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
     </row>
     <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -2150,8 +2152,8 @@
       <c r="J29" s="7">
         <v>1</v>
       </c>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="25"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -2183,8 +2185,8 @@
       <c r="J30" s="9">
         <v>1</v>
       </c>
-      <c r="K30" s="26"/>
-      <c r="L30" s="26"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="25"/>
     </row>
     <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -2201,23 +2203,23 @@
       <c r="E31" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F31" s="35" t="s">
+      <c r="F31" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="G31" s="38" t="s">
+      <c r="G31" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="H31" s="35" t="s">
+      <c r="H31" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="I31" s="38" t="s">
+      <c r="I31" s="37" t="s">
         <v>114</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
-      <c r="K31" s="26"/>
-      <c r="L31" s="26"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
     </row>
     <row r="32" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
@@ -2231,25 +2233,25 @@
       <c r="E32" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="F32" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="G32" s="36" t="s">
+      <c r="G32" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="H32" s="36" t="s">
+      <c r="H32" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="I32" s="39" t="s">
+      <c r="I32" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="J32" s="33"/>
-      <c r="K32" s="22" t="s">
+      <c r="J32" s="32"/>
+      <c r="K32" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="L32" s="26"/>
-    </row>
-    <row r="33" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L32" s="25"/>
+    </row>
+    <row r="33" spans="2:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f t="shared" si="1"/>
         <v>31</v>
@@ -2259,38 +2261,38 @@
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F33" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="F33" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="G33" s="37" t="s">
+      <c r="G33" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="H33" s="37" t="s">
+      <c r="H33" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="I33" s="40" t="s">
+      <c r="I33" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="J33" s="34"/>
-      <c r="K33" s="29" t="s">
-        <v>153</v>
-      </c>
-      <c r="L33" s="28"/>
+      <c r="J33" s="33"/>
+      <c r="K33" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="L33" s="27"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="L37" s="23"/>
-      <c r="M37" s="24"/>
+      <c r="L37" s="22"/>
+      <c r="M37" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:J1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K11" r:id="rId1" xr:uid="{03266B9D-911B-4550-9416-FC47FB8879C8}"/>
-    <hyperlink ref="K32" r:id="rId2" xr:uid="{D1E8C578-5D82-4E69-90F3-A5AB52CCB2B0}"/>
-    <hyperlink ref="K33" r:id="rId3" xr:uid="{28FA24B7-C6E6-4A1C-8CB5-9C4689576AE3}"/>
+    <hyperlink ref="K11" r:id="rId1"/>
+    <hyperlink ref="K32" r:id="rId2"/>
+    <hyperlink ref="K33" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>

</xml_diff>